<commit_message>
Track RIFoundationSystem/RigidInclusion rename in diggs-schema
Companion to diggs-schema's rename (RIFoundationSystem -> RigidInclusionSystem,
RigidInclusion -> RIColumn). Four workbooks updated and regenerated:

- samplingFeatureTypes.xlsx: dictionary IDs themselves renamed, not just display
  text - rigid_inclusion -> ri_column, ri_foundation_system ->
  rigid_inclusion_system (gml:id, derived identifier URL, name, description).
- columnType.xlsx: 11 AssociatedElements/SourceElement bindings fixed from
  //diggs:RigidInclusion/diggs:columnType to //diggs:RIColumn/diggs:columnType -
  a live Occurrence xpath, not documentation; would otherwise silently point at
  a now-nonexistent element.
- installationMethod.xlsx, grout_inj_properties.xlsx: description-text
  cross-references updated to match.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/columnType.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/columnType.xlsx
@@ -985,7 +985,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Codes naming the rigid inclusion installation technique family, shared by the design/specification intent (diggs:RIColumnSpecification/columnType) and the as-built record (diggs:RigidInclusion/columnType) so that design and as-built do not drift into different vocabularies for the same concept. Derived from the eleven-value installationType list carried by the retired CMCArrayType sketch (diggs-schema commit 0254e97, RigidInclusions.xsd, pre-C4 retirement). The list is open: technique families proliferate under proprietary trade names and cannot be closed.</t>
+          <t>Codes naming the rigid inclusion installation technique family, shared by the design/specification intent (diggs:RIColumnSpecification/columnType) and the as-built record (diggs:RIColumn/columnType) so that design and as-built do not drift into different vocabularies for the same concept. Derived from the eleven-value installationType list carried by the retired CMCArrayType sketch (diggs-schema commit 0254e97, RigidInclusions.xsd, pre-C4 retirement). The list is open: technique families proliferate under proprietary trade names and cannot be closed.</t>
         </is>
       </c>
     </row>
@@ -1764,7 +1764,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>//diggs:RigidInclusion/diggs:columnType</t>
+          <t>//diggs:RIColumn/diggs:columnType</t>
         </is>
       </c>
     </row>
@@ -1796,7 +1796,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>//diggs:RigidInclusion/diggs:columnType</t>
+          <t>//diggs:RIColumn/diggs:columnType</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>//diggs:RigidInclusion/diggs:columnType</t>
+          <t>//diggs:RIColumn/diggs:columnType</t>
         </is>
       </c>
     </row>
@@ -1860,7 +1860,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>//diggs:RigidInclusion/diggs:columnType</t>
+          <t>//diggs:RIColumn/diggs:columnType</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>//diggs:RigidInclusion/diggs:columnType</t>
+          <t>//diggs:RIColumn/diggs:columnType</t>
         </is>
       </c>
     </row>
@@ -1924,7 +1924,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>//diggs:RigidInclusion/diggs:columnType</t>
+          <t>//diggs:RIColumn/diggs:columnType</t>
         </is>
       </c>
     </row>
@@ -1956,7 +1956,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>//diggs:RigidInclusion/diggs:columnType</t>
+          <t>//diggs:RIColumn/diggs:columnType</t>
         </is>
       </c>
     </row>
@@ -1988,7 +1988,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>//diggs:RigidInclusion/diggs:columnType</t>
+          <t>//diggs:RIColumn/diggs:columnType</t>
         </is>
       </c>
     </row>
@@ -2020,7 +2020,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>//diggs:RigidInclusion/diggs:columnType</t>
+          <t>//diggs:RIColumn/diggs:columnType</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>//diggs:RigidInclusion/diggs:columnType</t>
+          <t>//diggs:RIColumn/diggs:columnType</t>
         </is>
       </c>
     </row>
@@ -2084,7 +2084,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>//diggs:RigidInclusion/diggs:columnType</t>
+          <t>//diggs:RIColumn/diggs:columnType</t>
         </is>
       </c>
     </row>

</xml_diff>